<commit_message>
Update OT instructions vs staffing reconciliation for revised table
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fzf6tjtbJa5AjBFghmbkhb
</commit_message>
<xml_diff>
--- a/Сверка_ИОТ_и_ШР_20.10.2026.xlsx
+++ b/Сверка_ИОТ_и_ШР_20.10.2026.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итог" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сверка ШР" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пункты без работников в ШР" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Замечания к таблице ИОТ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Изменения в версии" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сверка ШР" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пункты без работников в ШР" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Замечания к таблице ИОТ" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Сверка ШР'!$A$1:$F$237</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Сверка ШР'!$A$1:$F$237</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -510,7 +511,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Сверка: Таблица инструкций по ОТ (45 пунктов) ↔ Штатная расстановка на 20.10.2026 (746 чел.)</t>
+          <t>Сверка: Таблица инструкций по ОТ (обновлённая версия, 45 пунктов) ↔ Штатная расстановка на 20.10.2026 (746 чел.)</t>
         </is>
       </c>
     </row>
@@ -635,6 +636,114 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Ячейка</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Было</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Стало</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Оценка</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>C264 (п.17 Маляр)</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>пусто</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>ИОТ-16</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Частично. Номер внесён не в ту графу; перечень ИОТ (графа D) пуст.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>C265 (п.18 Главный энергетик)</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>пусто</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>ИОТ-17</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Частично. Номер внесён не в ту графу; перечень ИОТ (графа D) пуст.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Остальные 2 258 ячеек</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>без изменений</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Все прочие замечания первой сверки сохраняются.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1487,7 +1596,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Пункт 17 «Маляр» есть, но программа инструктажа и перечень ИОТ не заполнены.</t>
+          <t>В обновлённой версии в графу «Программа инструктажа» (C264) внесено «ИОТ-16». Программа отсутствует, графа «Инструкции» (D) пустая, наименование ИОТ-16 не указано.</t>
         </is>
       </c>
     </row>
@@ -1515,7 +1624,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Пункт 17 «Маляр» есть, но программа инструктажа и перечень ИОТ не заполнены.</t>
+          <t>В обновлённой версии в графу «Программа инструктажа» (C264) внесено «ИОТ-16». Программа отсутствует, графа «Инструкции» (D) пустая, наименование ИОТ-16 не указано.</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1652,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Пункт 18 есть, программа и ИОТ не заполнены.</t>
+          <t>В обновлённой версии в графу «Программа инструктажа» (C265) внесено «ИОТ-17». Программа отсутствует, графа «Инструкции» (D) пустая, наименование ИОТ-17 не указано.</t>
         </is>
       </c>
     </row>
@@ -6589,7 +6698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6760,13 +6869,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6793,19 +6902,19 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>п.17 Маляр, п.18 Главный энергетик, п.23 Специалист по пожарной безопасности, п.25 Инженер по АиРЭО — нет программы и перечня ИОТ. По ШР по ним 6 чел.</t>
+          <t>п.23 Специалист по пожарной безопасности, п.25 Инженер по АиРЭО — нет программы и перечня ИОТ.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Дубли номеров ИОТ</t>
+          <t>Не дозаполнены пп.17, 18</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>ИОТ-76: «при работе на компрессорной установке» (D36) и «с грузоподъёмными механизмами, управляемыми с пола» (D200, D281).</t>
+          <t>п.17 Маляр: «ИОТ-16», п.18 Главный энергетик: «ИОТ-17» внесены в графу C «Программа инструктажа» вместо графы D «Инструкции». Нет: программы инструктажа, полного наименования ИОТ, перечня сопутствующих ИОТ (ИОТ-01, 90, 107, 109 и др., как в остальных пунктах). Для маляра по смыслу нужны ИОТ-48, 83, 114 (ЛВЖ/ЛКМ, химвещества, смешение красок).</t>
         </is>
       </c>
     </row>
@@ -6817,101 +6926,113 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>ИОТ-80: «по ремонту и зарядке аккумуляторов» (D37) и «при работе с аккумулятором» (D88 и др.).</t>
+          <t>ИОТ-76: «при работе на компрессорной установке» (D36) и «с грузоподъёмными механизмами, управляемыми с пола» (D200, D281).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Одна инструкция — два номера</t>
+          <t>Дубли номеров ИОТ</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>«При работе на компрессорной установке»: ИОТ-76 (D36) и ИОТ-85 (D523).</t>
+          <t>ИОТ-80: «по ремонту и зарядке аккумуляторов» (D37) и «при работе с аккумулятором» (D88 и др.).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Латиница в номерах</t>
+          <t>Одна инструкция — два номера</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>«ИOT» с латинскими O/T — 37 ячеек (D32, D37, D46, D49 … D345); C21 «OXPAHE»; D521 «пpecce». Мешает поиску/фильтрации.</t>
+          <t>«При работе на компрессорной установке»: ИОТ-76 (D36) и ИОТ-85 (D523).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Опечатки в графе «Должность»/«Программа»</t>
+          <t>Латиница в номерах</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>п.2 «СЛЕСАРь-РЕМОНТННК»; п.9 «КОНТРОЛЁРА» (падеж); п.22 «ЭКСПЛУАТПЦИИ»; п.31 «ПРОГРАМИСТ»; п.36 «СТЕКЛОПЛАСТИКОВЫЗ»; пп.41–44 «ВСЕХРАЗРЯДОВ».</t>
+          <t>«ИOT» с латинскими O/T — 37 ячеек (D32, D37, D46, D49 … D345); C21 «OXPAHE»; D521 «пpecce». Мешает поиску/фильтрации.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Опечатки в наименованиях ИОТ</t>
+          <t>Опечатки в графе «Должность»/«Программа»</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>ИОТ-58 «Инстрщция … шлифовальньж»; ИОТ-87 «охране руда»; «ввтполнении» (ИОТ-46); «проеду» вместо «проезду» (ИОТ-109).</t>
+          <t>п.2 «СЛЕСАРь-РЕМОНТННК»; п.9 «КОНТРОЛЁРА» (падеж); п.22 «ЭКСПЛУАТПЦИИ»; п.31 «ПРОГРАМИСТ»; п.36 «СТЕКЛОПЛАСТИКОВЫЗ»; пп.41–44 «ВСЕХРАЗРЯДОВ».</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Расхождение наименований</t>
+          <t>Опечатки в наименованиях ИОТ</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>п.41 «листогибочного» ↔ ИОТ-40 «листосгибочного»; п.37 «оператор станка ЧПУ» ↔ ШР «оператор станков с ЧПУ».</t>
+          <t>ИОТ-58 «Инстрщция … шлифовальньж»; ИОТ-87 «охране руда»; «ввтполнении» (ИОТ-46); «проеду» вместо «проезду» (ИОТ-109).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Формулировки пунктов уже ИОТ</t>
+          <t>Расхождение наименований</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>п.9 — только «контролёр ОТК», а ИОТ-10 «инженер (контролёр) ОТК всех категорий»; п.13 — только «реставратор», а ИОТ-12 включает ведущего специалиста по реставрации; п.30 — только «сторож», а ИОТ-29 включает оперативных дежурных.</t>
+          <t>п.41 «листогибочного» ↔ ИОТ-40 «листосгибочного»; п.37 «оператор станка ЧПУ» ↔ ШР «оператор станков с ЧПУ».</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Неиспользуемые номера</t>
+          <t>Формулировки пунктов уже ИОТ</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>В таблице не встречаются ИОТ-05, 16, 17, 22, 24 — проверить по реестру ИОТ (возможно, предназначены для пустых пп.17, 18, 23, 25).</t>
+          <t>п.9 — только «контролёр ОТК», а ИОТ-10 «инженер (контролёр) ОТК всех категорий»; п.13 — только «реставратор», а ИОТ-12 включает ведущего специалиста по реставрации; п.30 — только «сторож», а ИОТ-29 включает оперативных дежурных.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
+          <t>Неиспользуемые номера</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>В графе «Инструкции» не встречаются ИОТ-05, 22, 24 (ИОТ-16, 17 теперь указаны в пп.17, 18). Проверить по реестру: возможно, предназначены для пп.23, 25.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
           <t>Замечание к ШР</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>«Слесарь - сборщик 4 разряда» (ОП Казань, 3 чел.) записан с пробелами, остальные — «Слесарь-сборщик». Аналогично «Инженер - конструктор» / «Инженер-конструктор» — разнобой в справочнике должностей.</t>
         </is>

</xml_diff>